<commit_message>
data(unknowable-domain): G10-P3-B5 author complete workbooks
</commit_message>
<xml_diff>
--- a/config/unknowable-domain-generated/templates/UnknowableDomain.xlsx
+++ b/config/unknowable-domain-generated/templates/UnknowableDomain.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4206" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4202" uniqueCount="318">
   <si>
     <t>@table</t>
   </si>
@@ -894,7 +894,7 @@
     <t>UnknowableDomainTalent</t>
   </si>
   <si>
-    <t>62470d4a1c601bc1</t>
+    <t>9e50dde3cb2506f2</t>
   </si>
   <si>
     <t>cost_json</t>
@@ -918,7 +918,7 @@
     <t>UnknowableDomainUnlock</t>
   </si>
   <si>
-    <t>d9e79e9f8fd98b2f</t>
+    <t>22e27aa55c64e617</t>
   </si>
   <si>
     <t>finish_condition_id</t>
@@ -948,7 +948,7 @@
     <t>UnknowableDomainMazeBuff</t>
   </si>
   <si>
-    <t>a8e702cdcac71c18</t>
+    <t>e97754352aab9a30</t>
   </si>
   <si>
     <t>series</t>
@@ -12035,8 +12035,7 @@
     <col min="15" max="17" width="12.7109375" style="5" customWidth="1"/>
     <col min="18" max="18" width="22.7109375" style="5" customWidth="1"/>
     <col min="19" max="19" width="23.7109375" style="5" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" style="5" customWidth="1"/>
-    <col min="21" max="21" width="22.7109375" style="5" customWidth="1"/>
+    <col min="20" max="21" width="22.7109375" style="5" customWidth="1"/>
     <col min="22" max="22" width="14.7109375" style="5" customWidth="1"/>
     <col min="23" max="23" width="17.7109375" style="5" customWidth="1"/>
     <col min="24" max="24" width="16.7109375" style="5" customWidth="1"/>
@@ -12281,7 +12280,7 @@
         <v>32</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="U4" s="5" t="s">
         <v>32</v>
@@ -12423,7 +12422,7 @@
         <v>66</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>79</v>
+        <v>45</v>
       </c>
       <c r="U6" s="5" t="s">
         <v>47</v>
@@ -12505,7 +12504,7 @@
     <col min="17" max="17" width="12.7109375" style="5" customWidth="1"/>
     <col min="18" max="18" width="19.7109375" style="5" customWidth="1"/>
     <col min="19" max="19" width="24.7109375" style="5" customWidth="1"/>
-    <col min="20" max="20" width="14.7109375" style="5" customWidth="1"/>
+    <col min="20" max="20" width="16.7109375" style="5" customWidth="1"/>
     <col min="21" max="21" width="17.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -12730,10 +12729,10 @@
         <v>36</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:21">
@@ -12851,12 +12850,8 @@
       <c r="S6" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="T6" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="U6" s="5" t="s">
-        <v>44</v>
-      </c>
+      <c r="T6" s="5"/>
+      <c r="U6" s="5"/>
     </row>
     <row r="7" spans="1:21" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
@@ -13354,7 +13349,8 @@
     <col min="13" max="14" width="22.7109375" style="5" customWidth="1"/>
     <col min="15" max="20" width="12.7109375" style="5" customWidth="1"/>
     <col min="21" max="21" width="15.7109375" style="5" customWidth="1"/>
-    <col min="22" max="23" width="14.7109375" style="5" customWidth="1"/>
+    <col min="22" max="22" width="14.7109375" style="5" customWidth="1"/>
+    <col min="23" max="23" width="16.7109375" style="5" customWidth="1"/>
     <col min="24" max="25" width="17.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -13612,10 +13608,10 @@
         <v>32</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="X4" s="5" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="Y4" s="5" t="s">
         <v>32</v>
@@ -13759,12 +13755,8 @@
       <c r="V6" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="W6" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="X6" s="5" t="s">
-        <v>44</v>
-      </c>
+      <c r="W6" s="5"/>
+      <c r="X6" s="5"/>
       <c r="Y6" s="5" t="s">
         <v>66</v>
       </c>

</xml_diff>

<commit_message>
data(unknowable-domain): G10-P3-B6 verify sora and visual qa
</commit_message>
<xml_diff>
--- a/config/unknowable-domain-generated/templates/UnknowableDomain.xlsx
+++ b/config/unknowable-domain-generated/templates/UnknowableDomain.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4202" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4202" uniqueCount="319">
   <si>
     <t>@table</t>
   </si>
@@ -312,7 +312,7 @@
     <t>UnknowableDomainLayer</t>
   </si>
   <si>
-    <t>a8baee40785b3c7e</t>
+    <t>6c58b501afa3d532</t>
   </si>
   <si>
     <t>layer_number</t>
@@ -324,28 +324,31 @@
     <t>carry_policy</t>
   </si>
   <si>
+    <t>range=0..1000</t>
+  </si>
+  <si>
+    <t>UnknowableDomainLayerRoom</t>
+  </si>
+  <si>
+    <t>24b2fbc5c2946f5e</t>
+  </si>
+  <si>
+    <t>layer_id</t>
+  </si>
+  <si>
+    <t>ordinal</t>
+  </si>
+  <si>
+    <t>room_pool_ids</t>
+  </si>
+  <si>
+    <t>room_pool_resolution</t>
+  </si>
+  <si>
+    <t>ref&lt;UnknowableDomainLayer.id&gt;</t>
+  </si>
+  <si>
     <t>range=0..100</t>
-  </si>
-  <si>
-    <t>UnknowableDomainLayerRoom</t>
-  </si>
-  <si>
-    <t>24b2fbc5c2946f5e</t>
-  </si>
-  <si>
-    <t>layer_id</t>
-  </si>
-  <si>
-    <t>ordinal</t>
-  </si>
-  <si>
-    <t>room_pool_ids</t>
-  </si>
-  <si>
-    <t>room_pool_resolution</t>
-  </si>
-  <si>
-    <t>ref&lt;UnknowableDomainLayer.id&gt;</t>
   </si>
   <si>
     <t>UnknowableDomainRoom</t>
@@ -1841,7 +1844,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -1865,7 +1868,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="24" customHeight="1">
@@ -1915,31 +1918,31 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>26</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:24">
@@ -1989,31 +1992,31 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="T3" s="5" t="s">
         <v>26</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:24">
@@ -2216,16 +2219,16 @@
       </c>
       <c r="T6" s="5"/>
       <c r="U6" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="V6" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="X6" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="42" customHeight="1">
@@ -2306,7 +2309,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2330,7 +2333,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="24" customHeight="1">
@@ -2380,31 +2383,31 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>82</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:24">
@@ -2454,31 +2457,31 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>82</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:24">
@@ -2528,7 +2531,7 @@
         <v>32</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>32</v>
@@ -2543,7 +2546,7 @@
         <v>63</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="V4" s="5" t="s">
         <v>32</v>
@@ -2674,23 +2677,23 @@
         <v>64</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="S6" s="5" t="s">
         <v>64</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="U6" s="5"/>
       <c r="V6" s="5" t="s">
         <v>47</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="X6" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="42" customHeight="1">
@@ -2775,7 +2778,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2799,7 +2802,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:28" ht="24" customHeight="1">
@@ -2849,43 +2852,43 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="Y2" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Z2" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="AA2" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:28">
@@ -2935,43 +2938,43 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="Y3" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Z3" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="AA3" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="AB3" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:28">
@@ -3021,10 +3024,10 @@
         <v>32</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>32</v>
@@ -3192,10 +3195,10 @@
         <v>66</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="U6" s="5" t="s">
         <v>47</v>
@@ -3299,7 +3302,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3323,7 +3326,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="24" customHeight="1">
@@ -3373,28 +3376,28 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>95</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:23">
@@ -3444,28 +3447,28 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="T3" s="5" t="s">
         <v>95</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -3515,13 +3518,13 @@
         <v>32</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="S4" s="5" t="s">
         <v>32</v>
@@ -3657,7 +3660,7 @@
         <v>66</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="U6" s="5" t="s">
         <v>66</v>
@@ -3742,7 +3745,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3766,7 +3769,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="24" customHeight="1">
@@ -4071,7 +4074,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4095,7 +4098,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:31" ht="24" customHeight="1">
@@ -4145,52 +4148,52 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>82</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="Y2" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="Z2" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AA2" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AC2" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AD2" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AE2" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:31">
@@ -4240,52 +4243,52 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="R3" s="5" t="s">
         <v>82</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="Y3" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="Z3" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AA3" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AB3" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AC3" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AD3" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AE3" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:31">
@@ -4338,7 +4341,7 @@
         <v>32</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>32</v>
@@ -4538,7 +4541,7 @@
         <v>66</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="X6" s="5" t="s">
         <v>65</v>
@@ -4647,7 +4650,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4671,7 +4674,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="24" customHeight="1">
@@ -4721,19 +4724,19 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="U2" s="3" t="s">
         <v>95</v>
@@ -4742,7 +4745,7 @@
         <v>54</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:23">
@@ -4792,19 +4795,19 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="U3" s="5" t="s">
         <v>95</v>
@@ -4813,7 +4816,7 @@
         <v>54</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -4863,13 +4866,13 @@
         <v>32</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>32</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="S4" s="5" t="s">
         <v>32</v>
@@ -5010,7 +5013,7 @@
         <v>46</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="V6" s="5" t="s">
         <v>66</v>
@@ -5094,7 +5097,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5118,7 +5121,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -5168,19 +5171,19 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -5230,19 +5233,19 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -5422,7 +5425,7 @@
         <v>64</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="42" customHeight="1">
@@ -5497,7 +5500,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5521,7 +5524,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="24" customHeight="1">
@@ -5571,28 +5574,28 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R2" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="U2" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="S2" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>141</v>
-      </c>
       <c r="V2" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="3" spans="1:23">
@@ -5642,28 +5645,28 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R3" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="U3" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="S3" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="T3" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>141</v>
-      </c>
       <c r="V3" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -5713,13 +5716,13 @@
         <v>32</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="S4" s="5" t="s">
         <v>63</v>
@@ -5852,13 +5855,13 @@
       <c r="Q6" s="5"/>
       <c r="R6" s="5"/>
       <c r="S6" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="T6" s="5" t="s">
         <v>47</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="V6" s="5" t="s">
         <v>66</v>
@@ -5941,7 +5944,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -5965,7 +5968,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="24" customHeight="1">
@@ -6015,22 +6018,22 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -6080,22 +6083,22 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -6892,7 +6895,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -6916,7 +6919,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="24" customHeight="1">
@@ -6966,22 +6969,22 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>54</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -7031,22 +7034,22 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>54</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -7096,7 +7099,7 @@
         <v>32</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>32</v>
@@ -7111,7 +7114,7 @@
         <v>63</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5" spans="1:21">
@@ -7230,7 +7233,7 @@
         <v>66</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="U6" s="5"/>
     </row>
@@ -7308,7 +7311,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7332,7 +7335,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="24" customHeight="1">
@@ -7382,28 +7385,28 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" spans="1:23">
@@ -7453,28 +7456,28 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -7524,7 +7527,7 @@
         <v>32</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>36</v>
@@ -7758,7 +7761,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -7782,7 +7785,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="24" customHeight="1">
@@ -7832,34 +7835,34 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="Y2" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -7909,34 +7912,34 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="Y3" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -8137,7 +8140,7 @@
         <v>42</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="R6" s="5" t="s">
         <v>47</v>
@@ -8239,7 +8242,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -8263,7 +8266,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="24" customHeight="1">
@@ -8313,28 +8316,28 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:23">
@@ -8384,28 +8387,28 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -8603,7 +8606,7 @@
         <v>66</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="U6" s="5" t="s">
         <v>47</v>
@@ -8689,7 +8692,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -8713,7 +8716,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="24" customHeight="1">
@@ -8763,31 +8766,31 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:24">
@@ -8837,31 +8840,31 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:24">
@@ -9150,7 +9153,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -9174,7 +9177,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -9224,13 +9227,13 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>54</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -9280,13 +9283,13 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>54</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -9442,7 +9445,7 @@
         <v>64</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>66</v>
@@ -9520,7 +9523,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -9544,7 +9547,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="24" customHeight="1">
@@ -9594,22 +9597,22 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -9659,22 +9662,22 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -9739,7 +9742,7 @@
         <v>32</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" spans="1:21">
@@ -9935,7 +9938,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -9959,7 +9962,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -10009,19 +10012,19 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -10071,19 +10074,19 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -10145,7 +10148,7 @@
         <v>32</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -10331,7 +10334,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -10355,7 +10358,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -10405,16 +10408,16 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>83</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -10464,16 +10467,16 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>83</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -10717,7 +10720,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -10741,7 +10744,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="24" customHeight="1">
@@ -10791,31 +10794,31 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="V2" s="3" t="s">
         <v>54</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:24">
@@ -10865,31 +10868,31 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="V3" s="5" t="s">
         <v>54</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:24">
@@ -11659,7 +11662,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -11683,7 +11686,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -11733,16 +11736,16 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -11792,16 +11795,16 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -12046,7 +12049,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -12070,7 +12073,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="24" customHeight="1">
@@ -12123,28 +12126,28 @@
         <v>82</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="3" spans="1:24">
@@ -12197,28 +12200,28 @@
         <v>82</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:24">
@@ -12513,7 +12516,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -12537,7 +12540,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="24" customHeight="1">
@@ -12587,22 +12590,22 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:21">
@@ -12652,22 +12655,22 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:21">
@@ -12717,7 +12720,7 @@
         <v>32</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>32</v>
@@ -12926,7 +12929,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -12950,7 +12953,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="24" customHeight="1">
@@ -13000,25 +13003,25 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>83</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="T2" s="3" t="s">
         <v>59</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -13068,25 +13071,25 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>83</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="T3" s="5" t="s">
         <v>59</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -13359,7 +13362,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -13383,7 +13386,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="24" customHeight="1">
@@ -13433,34 +13436,34 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>82</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="U2" s="3" t="s">
         <v>83</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="Y2" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -13510,34 +13513,34 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="R3" s="5" t="s">
         <v>82</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="U3" s="5" t="s">
         <v>83</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="Y3" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -13738,7 +13741,7 @@
         <v>42</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="R6" s="5" t="s">
         <v>64</v>
@@ -13833,7 +13836,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -13857,7 +13860,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -13907,19 +13910,19 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -13969,19 +13972,19 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -14158,7 +14161,7 @@
         <v>64</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="T6" s="5" t="s">
         <v>45</v>
@@ -14233,7 +14236,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -14257,7 +14260,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -14304,22 +14307,22 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>24</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -14366,22 +14369,22 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="P3" s="5" t="s">
         <v>24</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -14443,7 +14446,7 @@
         <v>32</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -15347,9 +15350,9 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: ExactStructured, ExactPublicText, Observed, ApproximateFromReleasedText, ProjectPolicy" promptTitle="UnknowableEvidenceQuality enum" prompt="Select a value from the dropdown." sqref="L8:L1007">
       <formula1>"ExactStructured,ExactPublicText,Observed,ApproximateFromReleasedText,ProjectPolicy"</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 0 to 100." promptTitle="Integer range" prompt="Enter an integer from 0 to 100." sqref="P8:P1007">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 0 to 1000." promptTitle="Integer range" prompt="Enter an integer from 0 to 1000." sqref="P8:P1007">
       <formula1>0</formula1>
-      <formula2>100</formula2>
+      <formula2>1000</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15687,7 +15690,7 @@
       </c>
       <c r="P6" s="5"/>
       <c r="Q6" s="5" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="R6" s="5" t="s">
         <v>45</v>
@@ -15767,7 +15770,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -15791,7 +15794,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -15841,16 +15844,16 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -15900,16 +15903,16 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -16151,7 +16154,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -16175,7 +16178,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -16222,22 +16225,22 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -16284,22 +16287,22 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -16346,7 +16349,7 @@
         <v>36</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="P4" s="5" t="s">
         <v>32</v>
@@ -16550,7 +16553,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -16574,7 +16577,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="24" customHeight="1">
@@ -16624,25 +16627,25 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -16692,25 +16695,25 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -16906,7 +16909,7 @@
         <v>42</v>
       </c>
       <c r="V6" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:22" ht="42" customHeight="1">

</xml_diff>